<commit_message>
ajuste en la ventana
</commit_message>
<xml_diff>
--- a/analysis_tools/agent_rewards_data.xlsx
+++ b/analysis_tools/agent_rewards_data.xlsx
@@ -30447,19 +30447,19 @@
         <v>1499</v>
       </c>
       <c r="B1501" t="n">
-        <v>125.7100000000001</v>
+        <v>154.5060000000001</v>
       </c>
       <c r="C1501" t="n">
-        <v>12.7</v>
+        <v>39.75</v>
       </c>
       <c r="D1501" t="n">
         <v>7</v>
       </c>
       <c r="E1501" t="n">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="F1501" t="n">
-        <v>23</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -60493,19 +60493,19 @@
         <v>1499</v>
       </c>
       <c r="B1501" t="n">
-        <v>123753.6</v>
+        <v>123782.396</v>
       </c>
       <c r="C1501" t="n">
-        <v>6507.050000000001</v>
+        <v>6534.100000000001</v>
       </c>
       <c r="D1501" t="n">
         <v>4826</v>
       </c>
       <c r="E1501" t="n">
-        <v>45335</v>
+        <v>45366</v>
       </c>
       <c r="F1501" t="n">
-        <v>14622</v>
+        <v>14646</v>
       </c>
     </row>
   </sheetData>
@@ -60561,10 +60561,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>82.502</v>
+        <v>82.52200000000001</v>
       </c>
       <c r="C2" t="n">
-        <v>93.09999999999999</v>
+        <v>93.111</v>
       </c>
       <c r="D2" t="n">
         <v>-118.228</v>
@@ -60573,7 +60573,7 @@
         <v>343.126</v>
       </c>
       <c r="F2" t="n">
-        <v>123753.6</v>
+        <v>123782.396</v>
       </c>
     </row>
     <row r="3">
@@ -60583,19 +60583,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4.338</v>
+        <v>4.356</v>
       </c>
       <c r="C3" t="n">
-        <v>6.383</v>
+        <v>6.444</v>
       </c>
       <c r="D3" t="n">
         <v>-16.3</v>
       </c>
       <c r="E3" t="n">
-        <v>17.05</v>
+        <v>39.75</v>
       </c>
       <c r="F3" t="n">
-        <v>6507.05</v>
+        <v>6534.1</v>
       </c>
     </row>
     <row r="4">
@@ -60627,19 +60627,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>30.223</v>
+        <v>30.244</v>
       </c>
       <c r="C5" t="n">
-        <v>17.468</v>
+        <v>17.509</v>
       </c>
       <c r="D5" t="n">
         <v>-27</v>
       </c>
       <c r="E5" t="n">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="F5" t="n">
-        <v>45335</v>
+        <v>45366</v>
       </c>
     </row>
     <row r="6">
@@ -60649,19 +60649,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9.747999999999999</v>
+        <v>9.763999999999999</v>
       </c>
       <c r="C6" t="n">
-        <v>10.212</v>
+        <v>10.251</v>
       </c>
       <c r="D6" t="n">
         <v>-28</v>
       </c>
       <c r="E6" t="n">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="F6" t="n">
-        <v>14622</v>
+        <v>14646</v>
       </c>
     </row>
   </sheetData>

</xml_diff>